<commit_message>
strategy_grp2: control board — three named strategy rows, minaggr on all
Runs sheet, 7 -> 10 rows.

New and active (purpose D, note "From strategy_grp"): Middle, Agressive,
Calm — the production trio the design note calls for, differing in
priority_attribute (rank / spr100d / spr100d). All three carry
informational_attributes = future_minaggr20d, which is what pulls
longi_future_minaggr20d.csv into the run's frozen snapshot: the
measurement layer for the stop-out feature, now readable from a tick.

The six from_rank/parity template rows keep their settings but change
tickers_per_group 5 -> 3, priority_direction big_wins -> small_wins and
from_rank 1 -> -1; fr_best/fr_mid/fr_worst are deactivated, so only the
three named rows run.

Tracked deliberately despite the blanket *.xlsx ignore — this board is a
hand-edited input, and its structure is worth versioning.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/strategy_grp2/app/control/control_board.xlsx
+++ b/strategy_grp2/app/control/control_board.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Gandalf\sm-home\potentials\strategy_grp2\app\control\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B2F6D7-9E3E-47A6-936C-2B2A5A7A3F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{611E44D2-EB13-49F1-8FB8-1536C660A58A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="975" yWindow="495" windowWidth="24255" windowHeight="16005" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3195" yWindow="2340" windowWidth="25335" windowHeight="14775" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Runs" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="109">
   <si>
     <t>active</t>
   </si>
@@ -328,6 +328,27 @@
   </si>
   <si>
     <t>per1d,future_per5d,future_per10d,future_per20d</t>
+  </si>
+  <si>
+    <t>Middle</t>
+  </si>
+  <si>
+    <t>From strategy_grp</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>small_wins</t>
+  </si>
+  <si>
+    <t>Calm</t>
+  </si>
+  <si>
+    <t>Agressive</t>
+  </si>
+  <si>
+    <t>future_minaggr20d</t>
   </si>
 </sst>
 </file>
@@ -717,10 +738,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="20" width="18" customWidth="1"/>
+    <col min="1" max="1" width="6.42578125" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="22.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="6.140625" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" customWidth="1"/>
+    <col min="9" max="20" width="18" customWidth="1"/>
     <col min="21" max="21" width="55.42578125" customWidth="1"/>
     <col min="22" max="22" width="18" customWidth="1"/>
   </cols>
@@ -819,16 +848,16 @@
         <v>10</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O2" t="s">
         <v>28</v>
       </c>
       <c r="P2" t="s">
-        <v>27</v>
+        <v>105</v>
       </c>
       <c r="Q2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="R2">
         <v>5</v>
@@ -869,16 +898,16 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O3" t="s">
         <v>28</v>
       </c>
       <c r="P3" t="s">
-        <v>27</v>
+        <v>105</v>
       </c>
       <c r="Q3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="R3">
         <v>5</v>
@@ -922,16 +951,16 @@
         <v>3</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O4" t="s">
         <v>28</v>
       </c>
       <c r="P4" t="s">
-        <v>27</v>
+        <v>105</v>
       </c>
       <c r="Q4">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="R4">
         <v>5</v>
@@ -947,9 +976,6 @@
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>30</v>
-      </c>
       <c r="B5" t="s">
         <v>31</v>
       </c>
@@ -978,16 +1004,16 @@
         <v>10</v>
       </c>
       <c r="M5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O5" t="s">
         <v>28</v>
       </c>
       <c r="P5" t="s">
-        <v>27</v>
+        <v>105</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="R5">
         <v>5</v>
@@ -1006,9 +1032,6 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>30</v>
-      </c>
       <c r="B6" t="s">
         <v>31</v>
       </c>
@@ -1037,13 +1060,13 @@
         <v>10</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O6" t="s">
         <v>28</v>
       </c>
       <c r="P6" t="s">
-        <v>27</v>
+        <v>105</v>
       </c>
       <c r="Q6" t="s">
         <v>36</v>
@@ -1065,9 +1088,6 @@
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>30</v>
-      </c>
       <c r="B7" t="s">
         <v>31</v>
       </c>
@@ -1096,13 +1116,13 @@
         <v>10</v>
       </c>
       <c r="M7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O7" t="s">
         <v>28</v>
       </c>
       <c r="P7" t="s">
-        <v>27</v>
+        <v>105</v>
       </c>
       <c r="Q7">
         <v>-1</v>
@@ -1121,6 +1141,174 @@
       </c>
       <c r="V7" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" t="s">
+        <v>104</v>
+      </c>
+      <c r="I8" t="s">
+        <v>26</v>
+      </c>
+      <c r="J8" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8">
+        <v>0.1</v>
+      </c>
+      <c r="L8">
+        <v>10</v>
+      </c>
+      <c r="M8">
+        <v>4</v>
+      </c>
+      <c r="O8" t="s">
+        <v>75</v>
+      </c>
+      <c r="P8" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q8">
+        <v>-1</v>
+      </c>
+      <c r="R8">
+        <v>5</v>
+      </c>
+      <c r="S8">
+        <v>20</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>107</v>
+      </c>
+      <c r="D9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" t="s">
+        <v>104</v>
+      </c>
+      <c r="I9" t="s">
+        <v>26</v>
+      </c>
+      <c r="J9" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9">
+        <v>0.1</v>
+      </c>
+      <c r="L9">
+        <v>10</v>
+      </c>
+      <c r="M9">
+        <v>4</v>
+      </c>
+      <c r="O9" t="s">
+        <v>28</v>
+      </c>
+      <c r="P9" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q9">
+        <v>-1</v>
+      </c>
+      <c r="R9">
+        <v>5</v>
+      </c>
+      <c r="S9">
+        <v>20</v>
+      </c>
+      <c r="T9">
+        <v>0</v>
+      </c>
+      <c r="U9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" t="s">
+        <v>103</v>
+      </c>
+      <c r="E10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10">
+        <v>0.1</v>
+      </c>
+      <c r="L10">
+        <v>5</v>
+      </c>
+      <c r="M10">
+        <v>3</v>
+      </c>
+      <c r="O10" t="s">
+        <v>28</v>
+      </c>
+      <c r="P10" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q10">
+        <v>-1</v>
+      </c>
+      <c r="R10">
+        <v>5</v>
+      </c>
+      <c r="S10">
+        <v>20</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
strategy_grp2: tickers_per_group/stop_loss recolored to step 2; board updates
param_spec.py: tickers_per_group and stop_loss both decide how the priority
list is drawn from/exited, same as post_filter/from_rank/priority_attribute
-- moved from steps 1/3 to step 2 so header colour (already changed by hand
on the board) matches on any future --make-board regeneration. Pure
cosmetic/legend change, step is never read for pipeline logic.

control_board.xlsx: SM's own edits this session (header recolour, per1d
post_filter correction on the NY rows, new US+post-filter comparison rows).
</commit_message>
<xml_diff>
--- a/strategy_grp2/app/control/control_board.xlsx
+++ b/strategy_grp2/app/control/control_board.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Gandalf\sm-home\potentials\strategy_grp2\app\control\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87AD1477-BFB0-43D2-96E6-26118D0ADD17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1190B29A-56A1-40F1-94DA-0AF12E0EA7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="225" yWindow="420" windowWidth="28305" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20145" yWindow="2115" windowWidth="27345" windowHeight="15165" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Runs" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="128">
   <si>
     <t>active</t>
   </si>
@@ -117,15 +117,9 @@
     <t>small_wins</t>
   </si>
   <si>
-    <t>per1d,future_per5d,future_per10d,future_per20d</t>
-  </si>
-  <si>
     <t>spr100d</t>
   </si>
   <si>
-    <t>conf_GICS</t>
-  </si>
-  <si>
     <t>Stamdata.Sector2</t>
   </si>
   <si>
@@ -373,6 +367,45 @@
   </si>
   <si>
     <t>Candidate pool (by label, comma-separated) for selection-skill scoring. Blank = every other active D-purpose row.</t>
+  </si>
+  <si>
+    <t>per1d</t>
+  </si>
+  <si>
+    <t>Stamdata.GICS .and. Stamdata.Zone='NY'</t>
+  </si>
+  <si>
+    <t>Longi.per1d&gt;0</t>
+  </si>
+  <si>
+    <t>4 (-1) NY</t>
+  </si>
+  <si>
+    <t>4 (-1) NY post-filter</t>
+  </si>
+  <si>
+    <t>5 (-1) NY</t>
+  </si>
+  <si>
+    <t>5 (-1) NY post-filter</t>
+  </si>
+  <si>
+    <t>Stamdata.Sector2 .and. Stamdata.Zone='NY'</t>
+  </si>
+  <si>
+    <t>11 (-1) NY</t>
+  </si>
+  <si>
+    <t>12 (-1) NY</t>
+  </si>
+  <si>
+    <t>per1d,spr100d</t>
+  </si>
+  <si>
+    <t>Longi.spr100d&lt;20</t>
+  </si>
+  <si>
+    <t>Longi.spr100d&lt;50</t>
   </si>
 </sst>
 </file>
@@ -391,16 +424,16 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -448,6 +481,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -461,7 +500,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -474,7 +513,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -777,10 +818,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W18"/>
+  <dimension ref="A1:W25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="20" width="18" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" customWidth="1"/>
+    <col min="3" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="39.140625" customWidth="1"/>
+    <col min="6" max="6" width="7.140625" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" customWidth="1"/>
+    <col min="8" max="16" width="18" customWidth="1"/>
+    <col min="17" max="17" width="10.5703125" customWidth="1"/>
+    <col min="18" max="20" width="18" customWidth="1"/>
     <col min="21" max="21" width="48.42578125" customWidth="1"/>
     <col min="22" max="23" width="18" customWidth="1"/>
   </cols>
@@ -822,7 +871,7 @@
       <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="10" t="s">
+      <c r="M1" s="4" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="4" t="s">
@@ -837,7 +886,7 @@
       <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="5" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="5" t="s">
@@ -860,6 +909,9 @@
       <c r="B2" t="s">
         <v>24</v>
       </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
       <c r="E2" t="s">
         <v>25</v>
       </c>
@@ -900,122 +952,117 @@
         <v>0</v>
       </c>
       <c r="U2" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="V2">
-        <v>-10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="9" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" t="s">
+        <v>28</v>
+      </c>
+      <c r="K3">
+        <v>0.1</v>
+      </c>
+      <c r="L3">
+        <v>10</v>
+      </c>
+      <c r="M3">
+        <v>3</v>
+      </c>
+      <c r="O3" t="s">
+        <v>27</v>
+      </c>
+      <c r="P3" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q3">
         <v>1</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="R3">
+        <v>5</v>
+      </c>
+      <c r="S3">
+        <v>20</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3" t="s">
+        <v>115</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="str">
+        <f>C3 &amp; " + stop "&amp;V4</f>
+        <v>2 + stop -20</v>
+      </c>
+      <c r="E4" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F4" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3" s="9">
+      <c r="I4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4">
         <v>0.1</v>
       </c>
-      <c r="L3" s="9">
+      <c r="L4">
         <v>10</v>
       </c>
-      <c r="M3" s="9">
-        <v>3</v>
-      </c>
-      <c r="O3" s="9" t="s">
+      <c r="M4">
+        <v>3</v>
+      </c>
+      <c r="O4" t="s">
         <v>27</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="P4" t="s">
         <v>28</v>
       </c>
-      <c r="Q3" s="9">
-        <v>-1</v>
-      </c>
-      <c r="R3" s="9">
-        <v>5</v>
-      </c>
-      <c r="S3" s="9">
+      <c r="Q4">
+        <v>1</v>
+      </c>
+      <c r="R4">
+        <v>5</v>
+      </c>
+      <c r="S4">
         <v>20</v>
       </c>
-      <c r="T3" s="9">
-        <v>0</v>
-      </c>
-      <c r="U3" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="V3" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="9">
-        <v>2</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K4" s="9">
-        <v>0.1</v>
-      </c>
-      <c r="L4" s="9">
-        <v>10</v>
-      </c>
-      <c r="M4" s="9">
-        <v>3</v>
-      </c>
-      <c r="O4" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="P4" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q4" s="9">
-        <v>-1</v>
-      </c>
-      <c r="R4" s="9">
-        <v>5</v>
-      </c>
-      <c r="S4" s="9">
-        <v>20</v>
-      </c>
-      <c r="T4" s="9">
-        <v>0</v>
-      </c>
-      <c r="U4" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="V4" s="9">
-        <v>0</v>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4" t="s">
+        <v>115</v>
+      </c>
+      <c r="V4">
+        <v>-20</v>
       </c>
     </row>
     <row r="5" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -1025,12 +1072,11 @@
       <c r="B5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="9" t="str">
-        <f>C4 &amp; " + stop "&amp;V5</f>
-        <v>2 + stop -20</v>
+      <c r="C5" s="9" t="s">
+        <v>118</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>26</v>
@@ -1048,10 +1094,11 @@
         <v>10</v>
       </c>
       <c r="M5" s="9">
-        <v>3</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="N5" s="10"/>
       <c r="O5" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="P5" s="9" t="s">
         <v>30</v>
@@ -1069,10 +1116,7 @@
         <v>0</v>
       </c>
       <c r="U5" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="V5" s="9">
-        <v>-20</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -1082,11 +1126,11 @@
       <c r="B6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="9">
-        <v>3</v>
+      <c r="C6" s="9" t="s">
+        <v>118</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>26</v>
@@ -1104,10 +1148,13 @@
         <v>10</v>
       </c>
       <c r="M6" s="9">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="N6" s="10" t="s">
+        <v>126</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P6" s="9" t="s">
         <v>30</v>
@@ -1125,10 +1172,7 @@
         <v>0</v>
       </c>
       <c r="U6" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="V6" s="9">
-        <v>0</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -1138,12 +1182,11 @@
       <c r="B7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="9" t="str">
-        <f>C6 &amp; " + stop "&amp;V7</f>
-        <v>3 + stop -20</v>
+      <c r="C7" s="9" t="s">
+        <v>118</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>26</v>
@@ -1161,10 +1204,13 @@
         <v>10</v>
       </c>
       <c r="M7" s="9">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="N7" s="10" t="s">
+        <v>127</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P7" s="9" t="s">
         <v>30</v>
@@ -1182,433 +1228,339 @@
         <v>0</v>
       </c>
       <c r="U7" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="K8" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="L8" s="9">
+        <v>10</v>
+      </c>
+      <c r="M8" s="9">
+        <v>3</v>
+      </c>
+      <c r="N8" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="O8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="V7" s="9">
-        <v>-20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
+      <c r="P8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q8" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R8" s="9">
+        <v>5</v>
+      </c>
+      <c r="S8" s="9">
+        <v>20</v>
+      </c>
+      <c r="T8" s="9">
+        <v>0</v>
+      </c>
+      <c r="U8" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="C9" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I9" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J9" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="K8">
+      <c r="K9" s="9">
         <v>0.1</v>
       </c>
-      <c r="L8">
+      <c r="L9" s="9">
         <v>10</v>
       </c>
-      <c r="M8">
-        <v>3</v>
-      </c>
-      <c r="O8" t="s">
-        <v>33</v>
-      </c>
-      <c r="P8" t="s">
+      <c r="M9" s="9">
+        <v>3</v>
+      </c>
+      <c r="N9" s="10"/>
+      <c r="O9" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="P9" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q9" s="9">
+        <v>1</v>
+      </c>
+      <c r="R9" s="9">
+        <v>5</v>
+      </c>
+      <c r="S9" s="9">
+        <v>20</v>
+      </c>
+      <c r="T9" s="9">
+        <v>0</v>
+      </c>
+      <c r="U9" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="Q8">
+      <c r="K10" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="L10" s="9">
+        <v>10</v>
+      </c>
+      <c r="M10" s="9">
+        <v>3</v>
+      </c>
+      <c r="N10" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="O10" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="P10" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q10" s="9">
         <v>1</v>
       </c>
-      <c r="R8">
-        <v>5</v>
-      </c>
-      <c r="S8">
+      <c r="R10" s="9">
+        <v>5</v>
+      </c>
+      <c r="S10" s="9">
         <v>20</v>
       </c>
-      <c r="T8">
-        <v>0</v>
-      </c>
-      <c r="U8" t="s">
+      <c r="T10" s="9">
+        <v>0</v>
+      </c>
+      <c r="U10" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="N11" s="10"/>
+    </row>
+    <row r="12" spans="1:23" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="11">
+        <v>10</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="K12" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="L12" s="11">
+        <v>5</v>
+      </c>
+      <c r="M12" s="11">
+        <v>3</v>
+      </c>
+      <c r="O12" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="P12" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q12" s="11">
+        <v>1</v>
+      </c>
+      <c r="R12" s="11">
+        <v>5</v>
+      </c>
+      <c r="S12" s="11">
+        <v>20</v>
+      </c>
+      <c r="T12" s="11">
+        <v>0</v>
+      </c>
+      <c r="U12" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="V12" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="K13" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="L13" s="11">
+        <v>3</v>
+      </c>
+      <c r="M13" s="11">
+        <v>3</v>
+      </c>
+      <c r="N13" s="12"/>
+      <c r="O13" s="11" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
+      <c r="P13" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q13" s="11">
+        <v>-1</v>
+      </c>
+      <c r="R13" s="11">
+        <v>5</v>
+      </c>
+      <c r="S13" s="11">
+        <v>20</v>
+      </c>
+      <c r="T13" s="11">
+        <v>0</v>
+      </c>
+      <c r="U13" s="11" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="C14" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="F14" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I14" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J14" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="K9">
+      <c r="K14" s="11">
         <v>0.1</v>
       </c>
-      <c r="L9">
-        <v>5</v>
-      </c>
-      <c r="M9">
-        <v>3</v>
-      </c>
-      <c r="O9" t="s">
-        <v>29</v>
-      </c>
-      <c r="P9" t="s">
+      <c r="L14" s="11">
+        <v>3</v>
+      </c>
+      <c r="M14" s="11">
+        <v>3</v>
+      </c>
+      <c r="N14" s="12"/>
+      <c r="O14" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="P14" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="Q9">
+      <c r="Q14" s="11">
         <v>1</v>
       </c>
-      <c r="R9">
-        <v>5</v>
-      </c>
-      <c r="S9">
+      <c r="R14" s="11">
+        <v>5</v>
+      </c>
+      <c r="S14" s="11">
         <v>20</v>
       </c>
-      <c r="T9">
-        <v>0</v>
-      </c>
-      <c r="U9" t="s">
-        <v>31</v>
-      </c>
-      <c r="V9">
-        <v>-5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" t="s">
-        <v>34</v>
-      </c>
-      <c r="F10" t="s">
-        <v>26</v>
-      </c>
-      <c r="I10" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" t="s">
-        <v>28</v>
-      </c>
-      <c r="K10">
-        <v>0.1</v>
-      </c>
-      <c r="L10">
-        <v>5</v>
-      </c>
-      <c r="M10">
-        <v>3</v>
-      </c>
-      <c r="O10" t="s">
-        <v>32</v>
-      </c>
-      <c r="P10" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q10">
-        <v>1</v>
-      </c>
-      <c r="R10">
-        <v>5</v>
-      </c>
-      <c r="S10">
-        <v>20</v>
-      </c>
-      <c r="T10">
-        <v>0</v>
-      </c>
-      <c r="U10" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" t="s">
-        <v>34</v>
-      </c>
-      <c r="F11" t="s">
-        <v>26</v>
-      </c>
-      <c r="I11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J11" t="s">
-        <v>28</v>
-      </c>
-      <c r="K11">
-        <v>0.1</v>
-      </c>
-      <c r="L11">
-        <v>5</v>
-      </c>
-      <c r="M11">
-        <v>3</v>
-      </c>
-      <c r="O11" t="s">
-        <v>35</v>
-      </c>
-      <c r="P11" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q11">
-        <v>1</v>
-      </c>
-      <c r="R11">
-        <v>5</v>
-      </c>
-      <c r="S11">
-        <v>20</v>
-      </c>
-      <c r="T11">
-        <v>0</v>
-      </c>
-      <c r="U11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" t="s">
-        <v>36</v>
-      </c>
-      <c r="F12" t="s">
-        <v>26</v>
-      </c>
-      <c r="I12" t="s">
-        <v>27</v>
-      </c>
-      <c r="J12" t="s">
-        <v>28</v>
-      </c>
-      <c r="K12">
-        <v>0.1</v>
-      </c>
-      <c r="L12">
-        <v>3</v>
-      </c>
-      <c r="M12">
-        <v>3</v>
-      </c>
-      <c r="O12" t="s">
-        <v>35</v>
-      </c>
-      <c r="P12" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q12">
-        <v>1</v>
-      </c>
-      <c r="R12">
-        <v>5</v>
-      </c>
-      <c r="S12">
-        <v>20</v>
-      </c>
-      <c r="T12">
-        <v>0</v>
-      </c>
-      <c r="U12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" t="s">
-        <v>37</v>
-      </c>
-      <c r="D13" t="s">
-        <v>38</v>
-      </c>
-      <c r="E13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" t="s">
-        <v>26</v>
-      </c>
-      <c r="I13" t="s">
-        <v>27</v>
-      </c>
-      <c r="J13" t="s">
-        <v>28</v>
-      </c>
-      <c r="K13">
-        <v>0.1</v>
-      </c>
-      <c r="L13">
-        <v>10</v>
-      </c>
-      <c r="M13">
-        <v>3</v>
-      </c>
-      <c r="O13" t="s">
-        <v>32</v>
-      </c>
-      <c r="P13" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q13">
-        <v>1</v>
-      </c>
-      <c r="R13">
-        <v>5</v>
-      </c>
-      <c r="S13">
-        <v>20</v>
-      </c>
-      <c r="T13">
-        <v>0</v>
-      </c>
-      <c r="U13" t="s">
-        <v>31</v>
-      </c>
-      <c r="W13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" t="s">
-        <v>26</v>
-      </c>
-      <c r="I14" t="s">
-        <v>27</v>
-      </c>
-      <c r="J14" t="s">
-        <v>28</v>
-      </c>
-      <c r="K14">
-        <v>0.1</v>
-      </c>
-      <c r="L14">
-        <v>10</v>
-      </c>
-      <c r="M14">
-        <v>3</v>
-      </c>
-      <c r="O14" t="s">
-        <v>32</v>
-      </c>
-      <c r="P14" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q14">
-        <v>1</v>
-      </c>
-      <c r="R14">
-        <v>5</v>
-      </c>
-      <c r="S14">
-        <v>20</v>
-      </c>
-      <c r="T14">
-        <v>0</v>
-      </c>
-      <c r="U14" t="s">
-        <v>31</v>
-      </c>
-      <c r="W14" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" t="s">
-        <v>41</v>
-      </c>
-      <c r="D15" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" t="s">
-        <v>25</v>
-      </c>
-      <c r="F15" t="s">
-        <v>26</v>
-      </c>
-      <c r="I15" t="s">
-        <v>27</v>
-      </c>
-      <c r="J15" t="s">
-        <v>28</v>
-      </c>
-      <c r="K15">
-        <v>0.1</v>
-      </c>
-      <c r="L15">
-        <v>10</v>
-      </c>
-      <c r="M15">
-        <v>3</v>
-      </c>
-      <c r="O15" t="s">
-        <v>32</v>
-      </c>
-      <c r="P15" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q15">
-        <v>-1</v>
-      </c>
-      <c r="R15">
-        <v>5</v>
-      </c>
-      <c r="S15">
-        <v>20</v>
-      </c>
-      <c r="T15">
-        <v>0</v>
-      </c>
-      <c r="U15" t="s">
-        <v>31</v>
-      </c>
-      <c r="W15" t="s">
-        <v>39</v>
-      </c>
+      <c r="T14" s="11">
+        <v>0</v>
+      </c>
+      <c r="U14" s="11" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="N15" s="12"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>24</v>
       </c>
-      <c r="C16" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" t="s">
-        <v>43</v>
-      </c>
       <c r="E16" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="F16" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="I16" t="s">
         <v>27</v>
@@ -1620,10 +1572,10 @@
         <v>0.1</v>
       </c>
       <c r="L16">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O16" t="s">
         <v>29</v>
@@ -1632,7 +1584,7 @@
         <v>30</v>
       </c>
       <c r="Q16">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="R16">
         <v>5</v>
@@ -1644,24 +1596,21 @@
         <v>0</v>
       </c>
       <c r="U16" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" spans="2:21" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+      <c r="V16">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>24</v>
       </c>
-      <c r="C17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" t="s">
-        <v>43</v>
-      </c>
       <c r="E17" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="F17" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="I17" t="s">
         <v>27</v>
@@ -1673,19 +1622,19 @@
         <v>0.1</v>
       </c>
       <c r="L17">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P17" t="s">
         <v>30</v>
       </c>
       <c r="Q17">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="R17">
         <v>5</v>
@@ -1697,21 +1646,15 @@
         <v>0</v>
       </c>
       <c r="U17" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" spans="2:21" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>24</v>
       </c>
-      <c r="C18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" t="s">
-        <v>43</v>
-      </c>
       <c r="E18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F18" t="s">
         <v>26</v>
@@ -1732,10 +1675,10 @@
         <v>3</v>
       </c>
       <c r="O18" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="P18" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="Q18">
         <v>1</v>
@@ -1750,7 +1693,381 @@
         <v>0</v>
       </c>
       <c r="U18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" t="s">
+        <v>26</v>
+      </c>
+      <c r="I19" t="s">
+        <v>27</v>
+      </c>
+      <c r="J19" t="s">
+        <v>28</v>
+      </c>
+      <c r="K19">
+        <v>0.1</v>
+      </c>
+      <c r="L19">
+        <v>3</v>
+      </c>
+      <c r="M19">
+        <v>3</v>
+      </c>
+      <c r="O19" t="s">
+        <v>33</v>
+      </c>
+      <c r="P19" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q19">
+        <v>1</v>
+      </c>
+      <c r="R19">
+        <v>5</v>
+      </c>
+      <c r="S19">
+        <v>20</v>
+      </c>
+      <c r="T19">
+        <v>0</v>
+      </c>
+      <c r="U19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" t="s">
+        <v>26</v>
+      </c>
+      <c r="I20" t="s">
+        <v>27</v>
+      </c>
+      <c r="J20" t="s">
+        <v>28</v>
+      </c>
+      <c r="K20">
+        <v>0.1</v>
+      </c>
+      <c r="L20">
+        <v>10</v>
+      </c>
+      <c r="M20">
+        <v>3</v>
+      </c>
+      <c r="O20" t="s">
+        <v>31</v>
+      </c>
+      <c r="P20" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q20">
+        <v>1</v>
+      </c>
+      <c r="R20">
+        <v>5</v>
+      </c>
+      <c r="S20">
+        <v>20</v>
+      </c>
+      <c r="T20">
+        <v>0</v>
+      </c>
+      <c r="U20" t="s">
+        <v>115</v>
+      </c>
+      <c r="W20" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21" t="s">
+        <v>26</v>
+      </c>
+      <c r="I21" t="s">
+        <v>27</v>
+      </c>
+      <c r="J21" t="s">
+        <v>28</v>
+      </c>
+      <c r="K21">
+        <v>0.1</v>
+      </c>
+      <c r="L21">
+        <v>10</v>
+      </c>
+      <c r="M21">
+        <v>3</v>
+      </c>
+      <c r="O21" t="s">
+        <v>31</v>
+      </c>
+      <c r="P21" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q21">
+        <v>1</v>
+      </c>
+      <c r="R21">
+        <v>5</v>
+      </c>
+      <c r="S21">
+        <v>20</v>
+      </c>
+      <c r="T21">
+        <v>0</v>
+      </c>
+      <c r="U21" t="s">
+        <v>115</v>
+      </c>
+      <c r="W21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22" t="s">
+        <v>26</v>
+      </c>
+      <c r="I22" t="s">
+        <v>27</v>
+      </c>
+      <c r="J22" t="s">
+        <v>28</v>
+      </c>
+      <c r="K22">
+        <v>0.1</v>
+      </c>
+      <c r="L22">
+        <v>10</v>
+      </c>
+      <c r="M22">
+        <v>3</v>
+      </c>
+      <c r="O22" t="s">
+        <v>31</v>
+      </c>
+      <c r="P22" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q22">
+        <v>-1</v>
+      </c>
+      <c r="R22">
+        <v>5</v>
+      </c>
+      <c r="S22">
+        <v>20</v>
+      </c>
+      <c r="T22">
+        <v>0</v>
+      </c>
+      <c r="U22" t="s">
+        <v>115</v>
+      </c>
+      <c r="W22" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" t="s">
+        <v>41</v>
+      </c>
+      <c r="E23" t="s">
+        <v>25</v>
+      </c>
+      <c r="F23" t="s">
+        <v>42</v>
+      </c>
+      <c r="I23" t="s">
+        <v>27</v>
+      </c>
+      <c r="J23" t="s">
+        <v>28</v>
+      </c>
+      <c r="K23">
+        <v>0.1</v>
+      </c>
+      <c r="L23">
+        <v>10</v>
+      </c>
+      <c r="M23">
+        <v>4</v>
+      </c>
+      <c r="O23" t="s">
+        <v>29</v>
+      </c>
+      <c r="P23" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q23">
+        <v>-1</v>
+      </c>
+      <c r="R23">
+        <v>5</v>
+      </c>
+      <c r="S23">
+        <v>20</v>
+      </c>
+      <c r="T23">
+        <v>0</v>
+      </c>
+      <c r="U23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" t="s">
+        <v>42</v>
+      </c>
+      <c r="I24" t="s">
+        <v>27</v>
+      </c>
+      <c r="J24" t="s">
+        <v>28</v>
+      </c>
+      <c r="K24">
+        <v>0.1</v>
+      </c>
+      <c r="L24">
+        <v>10</v>
+      </c>
+      <c r="M24">
+        <v>4</v>
+      </c>
+      <c r="O24" t="s">
+        <v>31</v>
+      </c>
+      <c r="P24" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q24">
+        <v>-1</v>
+      </c>
+      <c r="R24">
+        <v>5</v>
+      </c>
+      <c r="S24">
+        <v>20</v>
+      </c>
+      <c r="T24">
+        <v>0</v>
+      </c>
+      <c r="U24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" t="s">
         <v>45</v>
+      </c>
+      <c r="D25" t="s">
+        <v>41</v>
+      </c>
+      <c r="E25" t="s">
+        <v>32</v>
+      </c>
+      <c r="F25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I25" t="s">
+        <v>27</v>
+      </c>
+      <c r="J25" t="s">
+        <v>28</v>
+      </c>
+      <c r="K25">
+        <v>0.1</v>
+      </c>
+      <c r="L25">
+        <v>5</v>
+      </c>
+      <c r="M25">
+        <v>3</v>
+      </c>
+      <c r="O25" t="s">
+        <v>33</v>
+      </c>
+      <c r="P25" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q25">
+        <v>1</v>
+      </c>
+      <c r="R25">
+        <v>5</v>
+      </c>
+      <c r="S25">
+        <v>20</v>
+      </c>
+      <c r="T25">
+        <v>0</v>
+      </c>
+      <c r="U25" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1771,90 +2088,90 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>48</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B3">
         <v>315</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B4">
         <v>63</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B5" t="b">
         <v>1</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B6">
         <v>3</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>61</v>
-      </c>
-      <c r="B7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B8">
         <v>5</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1877,22 +2194,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>70</v>
-      </c>
       <c r="F1" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1900,16 +2217,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" t="s">
         <v>71</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" s="8" t="s">
         <v>72</v>
-      </c>
-      <c r="D2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1917,19 +2234,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D3" t="s">
         <v>24</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1937,13 +2254,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1951,13 +2268,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>78</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1968,10 +2285,10 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1982,16 +2299,16 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D7" t="s">
         <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -2002,10 +2319,10 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2016,13 +2333,13 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>87</v>
-      </c>
-      <c r="D9" t="s">
-        <v>88</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2033,13 +2350,13 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D10" t="s">
         <v>29</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2050,13 +2367,13 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>91</v>
-      </c>
-      <c r="D11" t="s">
-        <v>92</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -2067,13 +2384,13 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -2084,13 +2401,13 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -2101,13 +2418,13 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F14" s="8" t="s">
         <v>96</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -2118,10 +2435,10 @@
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -2132,13 +2449,13 @@
         <v>2</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D16" t="s">
         <v>29</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -2149,13 +2466,13 @@
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D17" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -2169,10 +2486,10 @@
         <v>16</v>
       </c>
       <c r="D18" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -2183,13 +2500,13 @@
         <v>2</v>
       </c>
       <c r="C19" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D19" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -2200,16 +2517,16 @@
         <v>3</v>
       </c>
       <c r="C20" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
+        <v>104</v>
+      </c>
+      <c r="E20" t="s">
+        <v>105</v>
+      </c>
+      <c r="F20" s="8" t="s">
         <v>106</v>
-      </c>
-      <c r="E20" t="s">
-        <v>107</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -2220,13 +2537,13 @@
         <v>3</v>
       </c>
       <c r="C21" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D21" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -2237,13 +2554,13 @@
         <v>3</v>
       </c>
       <c r="C22" t="s">
+        <v>109</v>
+      </c>
+      <c r="D22" t="s">
+        <v>110</v>
+      </c>
+      <c r="F22" s="8" t="s">
         <v>111</v>
-      </c>
-      <c r="D22" t="s">
-        <v>112</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -2254,13 +2571,13 @@
         <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D23" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -2271,10 +2588,10 @@
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>